<commit_message>
Put in place emulation of the ESP32 FPGA interface in C#.
</commit_message>
<xml_diff>
--- a/Spreadsheets/BasicCalculations.xlsx
+++ b/Spreadsheets/BasicCalculations.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1773" uniqueCount="1138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1789" uniqueCount="1147">
   <si>
     <t>N stages required</t>
   </si>
@@ -3460,6 +3460,33 @@
   </si>
   <si>
     <t>(d/(2l))^2</t>
+  </si>
+  <si>
+    <t>IPC-2221 Track Thickness Calculation</t>
+  </si>
+  <si>
+    <t>Internal else External</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>Allowable rise in temperature</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cross-Sectional Area </t>
+  </si>
+  <si>
+    <t>mil^2</t>
+  </si>
+  <si>
+    <t>Thickness</t>
+  </si>
+  <si>
+    <t>RMS Current</t>
+  </si>
+  <si>
+    <t>Width</t>
   </si>
 </sst>
 </file>
@@ -3854,7 +3881,7 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3871,6 +3898,9 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3882,9 +3912,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -4738,15 +4765,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>3038475</xdr:colOff>
-      <xdr:row>950</xdr:row>
-      <xdr:rowOff>161925</xdr:rowOff>
+      <xdr:colOff>2514600</xdr:colOff>
+      <xdr:row>945</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>628954</xdr:colOff>
-      <xdr:row>954</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:colOff>105079</xdr:colOff>
+      <xdr:row>949</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4763,8 +4790,84 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6619875" y="181575075"/>
+          <a:off x="6096000" y="181403625"/>
           <a:ext cx="3686479" cy="638175"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>3829050</xdr:colOff>
+      <xdr:row>960</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1505260</xdr:colOff>
+      <xdr:row>966</xdr:row>
+      <xdr:rowOff>136</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="Picture 16"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7410450" y="184251600"/>
+          <a:ext cx="2219635" cy="971686"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>3800475</xdr:colOff>
+      <xdr:row>966</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>676473</xdr:colOff>
+      <xdr:row>970</xdr:row>
+      <xdr:rowOff>95363</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="20" name="Picture 19"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7381875" y="185270775"/>
+          <a:ext cx="1419423" cy="809738"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -7130,13 +7233,13 @@
       <c r="E111" t="s">
         <v>25</v>
       </c>
-      <c r="G111" s="74" t="s">
+      <c r="G111" s="80" t="s">
         <v>1013</v>
       </c>
-      <c r="H111" s="74"/>
-      <c r="I111" s="74"/>
-      <c r="J111" s="74"/>
-      <c r="K111" s="74"/>
+      <c r="H111" s="80"/>
+      <c r="I111" s="80"/>
+      <c r="J111" s="80"/>
+      <c r="K111" s="80"/>
     </row>
     <row r="112" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A112" s="75"/>
@@ -20116,35 +20219,35 @@
         <v>206</v>
       </c>
       <c r="G941">
-        <f>$E941</f>
+        <f t="shared" ref="G941:N941" si="86">$E941</f>
         <v>1.2566370614359173E-6</v>
       </c>
       <c r="H941">
-        <f>$E941</f>
+        <f t="shared" si="86"/>
         <v>1.2566370614359173E-6</v>
       </c>
       <c r="I941">
-        <f>$E941</f>
+        <f t="shared" si="86"/>
         <v>1.2566370614359173E-6</v>
       </c>
       <c r="J941">
-        <f>$E941</f>
+        <f t="shared" si="86"/>
         <v>1.2566370614359173E-6</v>
       </c>
       <c r="K941">
-        <f>$E941</f>
+        <f t="shared" si="86"/>
         <v>1.2566370614359173E-6</v>
       </c>
       <c r="L941">
-        <f>$E941</f>
+        <f t="shared" si="86"/>
         <v>1.2566370614359173E-6</v>
       </c>
       <c r="M941">
-        <f>$E941</f>
+        <f t="shared" si="86"/>
         <v>1.2566370614359173E-6</v>
       </c>
       <c r="N941">
-        <f>$E941</f>
+        <f t="shared" si="86"/>
         <v>1.2566370614359173E-6</v>
       </c>
     </row>
@@ -20242,35 +20345,35 @@
         <v>154</v>
       </c>
       <c r="G949">
-        <f t="shared" ref="F949:N949" si="86">(G941/(4*PI()))*(LN(G944+SQRT(1+G946)) - SQRT(1+G947)+G945)</f>
+        <f t="shared" ref="G949:N949" si="87">(G941/(4*PI()))*(LN(G944+SQRT(1+G946)) - SQRT(1+G947)+G945)</f>
         <v>-1.0000000000000001E-7</v>
       </c>
       <c r="H949">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>-1.0000000000000001E-7</v>
       </c>
       <c r="I949">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>-1.0000000000000001E-7</v>
       </c>
       <c r="J949">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>-1.0000000000000001E-7</v>
       </c>
       <c r="K949">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>-1.0000000000000001E-7</v>
       </c>
       <c r="L949">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>-1.0000000000000001E-7</v>
       </c>
       <c r="M949">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>-1.0000000000000001E-7</v>
       </c>
       <c r="N949">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>-1.0000000000000001E-7</v>
       </c>
     </row>
@@ -20289,7 +20392,7 @@
     </row>
     <row r="951" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A951" s="75"/>
-      <c r="B951" s="84" t="s">
+      <c r="B951" s="74" t="s">
         <v>1095</v>
       </c>
       <c r="C951" t="s">
@@ -20339,39 +20442,39 @@
         <v>2.096571294539476E-2</v>
       </c>
       <c r="F952" t="e">
-        <f t="shared" ref="F952:N952" si="87">F950*COS(F951)*F949</f>
+        <f t="shared" ref="F952:N952" si="88">F950*COS(F951)*F949</f>
         <v>#VALUE!</v>
       </c>
       <c r="G952">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>0</v>
       </c>
       <c r="H952">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>0</v>
       </c>
       <c r="I952">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>0</v>
       </c>
       <c r="J952">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>0</v>
       </c>
       <c r="K952">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>0</v>
       </c>
       <c r="L952">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>0</v>
       </c>
       <c r="M952">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>0</v>
       </c>
       <c r="N952">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>0</v>
       </c>
     </row>
@@ -20447,40 +20550,106 @@
     <row r="960" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A960" s="75"/>
     </row>
-    <row r="962" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A962" s="75"/>
-    </row>
-    <row r="963" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="962" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A962" s="75" t="s">
+        <v>1138</v>
+      </c>
+      <c r="B962" t="s">
+        <v>1139</v>
+      </c>
+      <c r="C962" t="s">
+        <v>1139</v>
+      </c>
+      <c r="E962" s="52" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="963" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A963" s="75"/>
-    </row>
-    <row r="964" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B963" t="s">
+        <v>511</v>
+      </c>
+      <c r="E963" s="27">
+        <f>IF(E962, 0.024, 0.048)</f>
+        <v>4.8000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="964" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A964" s="75"/>
-    </row>
-    <row r="965" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B964" t="s">
+        <v>1140</v>
+      </c>
+      <c r="C964" t="s">
+        <v>1145</v>
+      </c>
+      <c r="E964" s="52">
+        <f>22/SQRT(3)</f>
+        <v>12.701705922171767</v>
+      </c>
+      <c r="F964" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="965" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A965" s="75"/>
-    </row>
-    <row r="966" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B965" s="74" t="s">
+        <v>693</v>
+      </c>
+      <c r="C965" t="s">
+        <v>1141</v>
+      </c>
+      <c r="E965">
+        <v>10</v>
+      </c>
+      <c r="F965" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="966" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A966" s="75"/>
-    </row>
-    <row r="967" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="C966" t="s">
+        <v>1144</v>
+      </c>
+      <c r="E966">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="967" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A967" s="75"/>
-    </row>
-    <row r="968" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B967" t="s">
+        <v>20</v>
+      </c>
+      <c r="C967" t="s">
+        <v>1142</v>
+      </c>
+      <c r="E967">
+        <f>POWER(E964/(E963*POWER(E965, 0.44)), (1/0.725))</f>
+        <v>542.8119517712156</v>
+      </c>
+      <c r="F967" t="s">
+        <v>1143</v>
+      </c>
+    </row>
+    <row r="968" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A968" s="75"/>
+      <c r="C968" t="s">
+        <v>1146</v>
+      </c>
+      <c r="E968">
+        <f>E967/(E966*1.378*39.37)</f>
+        <v>5.0027036102653044</v>
+      </c>
+      <c r="F968" t="s">
+        <v>133</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="A940:A952"/>
-    <mergeCell ref="A954:A960"/>
-    <mergeCell ref="A962:A968"/>
-    <mergeCell ref="A892:A906"/>
-    <mergeCell ref="A568:A580"/>
-    <mergeCell ref="A581:A584"/>
-    <mergeCell ref="A781:A793"/>
-    <mergeCell ref="A695:A766"/>
-    <mergeCell ref="A653:A692"/>
-    <mergeCell ref="A799:A819"/>
-    <mergeCell ref="A821:A841"/>
+    <mergeCell ref="G111:K111"/>
+    <mergeCell ref="A99:A136"/>
+    <mergeCell ref="A196:A220"/>
+    <mergeCell ref="A167:A193"/>
+    <mergeCell ref="A138:A164"/>
     <mergeCell ref="A31:A59"/>
     <mergeCell ref="A858:A883"/>
     <mergeCell ref="A286:A337"/>
@@ -20497,16 +20666,22 @@
     <mergeCell ref="A844:A856"/>
     <mergeCell ref="A414:A454"/>
     <mergeCell ref="A456:A566"/>
+    <mergeCell ref="A940:A952"/>
+    <mergeCell ref="A954:A960"/>
+    <mergeCell ref="A962:A968"/>
+    <mergeCell ref="A892:A906"/>
+    <mergeCell ref="A568:A580"/>
+    <mergeCell ref="A581:A584"/>
+    <mergeCell ref="A781:A793"/>
+    <mergeCell ref="A695:A766"/>
+    <mergeCell ref="A653:A692"/>
+    <mergeCell ref="A799:A819"/>
+    <mergeCell ref="A821:A841"/>
     <mergeCell ref="A910:A912"/>
     <mergeCell ref="A915:A917"/>
     <mergeCell ref="A920:A922"/>
     <mergeCell ref="A925:A930"/>
     <mergeCell ref="A932:A937"/>
-    <mergeCell ref="G111:K111"/>
-    <mergeCell ref="A99:A136"/>
-    <mergeCell ref="A196:A220"/>
-    <mergeCell ref="A167:A193"/>
-    <mergeCell ref="A138:A164"/>
   </mergeCells>
   <conditionalFormatting sqref="D120">
     <cfRule type="cellIs" dxfId="11" priority="11" operator="notEqual">
@@ -20809,17 +20984,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="80" t="s">
+      <c r="A1" s="81" t="s">
         <v>149</v>
       </c>
-      <c r="B1" s="80"/>
+      <c r="B1" s="81"/>
     </row>
     <row r="18" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C18" s="81" t="s">
+      <c r="C18" s="82" t="s">
         <v>161</v>
       </c>
-      <c r="D18" s="82"/>
-      <c r="E18" s="83"/>
+      <c r="D18" s="83"/>
+      <c r="E18" s="84"/>
     </row>
     <row r="19" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C19" s="17" t="s">
@@ -21013,17 +21188,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="80" t="s">
+      <c r="A1" s="81" t="s">
         <v>160</v>
       </c>
-      <c r="B1" s="80"/>
+      <c r="B1" s="81"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B17" s="81" t="s">
+      <c r="B17" s="82" t="s">
         <v>161</v>
       </c>
-      <c r="C17" s="82"/>
-      <c r="D17" s="83"/>
+      <c r="C17" s="83"/>
+      <c r="D17" s="84"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B18" s="17" t="s">
@@ -21276,17 +21451,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="80" t="s">
+      <c r="A1" s="81" t="s">
         <v>167</v>
       </c>
-      <c r="B1" s="80"/>
+      <c r="B1" s="81"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B17" s="81" t="s">
+      <c r="B17" s="82" t="s">
         <v>161</v>
       </c>
-      <c r="C17" s="82"/>
-      <c r="D17" s="83"/>
+      <c r="C17" s="83"/>
+      <c r="D17" s="84"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B18" s="17" t="s">

</xml_diff>